<commit_message>
judgment: light-load advisory resets per-phase persistence clocks (follow-up fix) + comparison workbook tooling
- Judge._light_load_policy(t, out): 경부하 동안 세 상 내부 상태 SAFE·지속 시계 리셋 → 경부하 뒤 결상·과전류도 3 s 지속 규칙
  (검증 배치에서 8턴 장면이 무부하에서 넘겨받은 DANGER 로 지속 없이 위험 판정 → 수정). 테스트·judgment_basis §8·SESSION_LOG 갱신
- demo_integrated --verify_dir meta.json 에 git_commit 기록
- tools/verify/sim_vs_maxwell_xlsx.py(엑셀 9시트+차트 3, 역추정, FEM 민감도, 요약 md) + tests/test_sim_vs_maxwell_xlsx.py (로그 재실행 뒤 산출물 커밋)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/verification/sim_vs_analysis.xlsx
+++ b/docs/verification/sim_vs_analysis.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="대조표" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="이벤트" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="재계산" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="민감도" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="열" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대조표" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="이벤트" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="재계산" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="민감도" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="열" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,12 +33,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0B2"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -53,9 +58,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -500,7 +506,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>n=89</t>
+          <t>n=86</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -872,7 +878,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>n=89</t>
+          <t>n=83</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1370,7 +1376,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3.01</v>
+        <v>2.99</v>
       </c>
       <c r="D23" t="n">
         <v>3</v>
@@ -1426,7 +1432,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>n=87</t>
+          <t>n=88</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1876,7 +1882,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3.07</v>
+        <v>2.96</v>
       </c>
       <c r="D35" t="n">
         <v>3</v>
@@ -1932,7 +1938,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>n=88</t>
+          <t>n=89</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -1970,7 +1976,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>n=89</t>
+          <t>n=87</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2008,7 +2014,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>n=88</t>
+          <t>n=86</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2084,7 +2090,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>n=88</t>
+          <t>n=86</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2483,44 +2489,44 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>탐지 지연 [s] (주입 → 첫 상향, 지속 3 s 규칙)</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>itsc_8turn</t>
         </is>
       </c>
-      <c r="C50" t="n">
-        <v>3.07</v>
-      </c>
-      <c r="D50" t="n">
+      <c r="C50" s="2" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="D50" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E50" t="n">
+      <c r="E50" s="2" t="n">
         <v>0.2</v>
       </c>
-      <c r="F50">
+      <c r="F50" s="2">
         <f>(C50/D50-1)*100</f>
         <v/>
       </c>
-      <c r="G50">
+      <c r="G50" s="2">
         <f>IF(ABS(F50)&lt;=E50*100,"PASS","FAIL")</f>
         <v/>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>첫 DANGER</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>thresholds.yaml persistence_s</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
         <is>
           <t>rel</t>
         </is>
@@ -2550,7 +2556,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>n=89</t>
+          <t>n=88</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3012,7 +3018,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>n=90</t>
+          <t>n=88</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3522,7 +3528,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>n=88</t>
+          <t>n=86</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3972,7 +3978,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>3.03</v>
+        <v>2.96</v>
       </c>
       <c r="D85" t="n">
         <v>3</v>
@@ -4027,7 +4033,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>356 행</t>
+          <t>351 행</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4068,7 +4074,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>127 파형, 기본파 외 고조파 0</t>
+          <t>174 파형, 기본파 외 고조파 0</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -4310,11 +4316,11 @@
         <v>20</v>
       </c>
       <c r="C3" t="n">
-        <v>23.007</v>
+        <v>22.986</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{"WARN": 3.01}</t>
+          <t>{"WARN": 2.99}</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4343,11 +4349,11 @@
         <v>45</v>
       </c>
       <c r="D4" t="n">
-        <v>48.067</v>
+        <v>47.959</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>{"DANGER": 3.07}</t>
+          <t>{"DANGER": 2.96}</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -4376,11 +4382,11 @@
         <v>165</v>
       </c>
       <c r="D5" t="n">
-        <v>168.067</v>
+        <v>164.946</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>{"DANGER": 3.07}</t>
+          <t>{"DANGER": -0.05}</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -4469,11 +4475,11 @@
         <v>225</v>
       </c>
       <c r="C8" t="n">
-        <v>228.035</v>
+        <v>227.962</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>{"WARN": 3.03}</t>
+          <t>{"WARN": 2.96}</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -4578,7 +4584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G128"/>
+  <dimension ref="A1:G175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4688,19 +4694,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>waveform_0020.00_post_itsc_4turn.csv</t>
+          <t>waveform_0000.08_post_healthy.csv</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>itsc_4turn</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.07262299999999999</v>
+        <v>0.027</v>
       </c>
       <c r="E4" t="n">
-        <v>0.07262</v>
+        <v>0.027</v>
       </c>
       <c r="F4">
         <f>(D4/E4-1)*100</f>
@@ -4719,19 +4725,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>waveform_0020.00_pre_healthy.csv</t>
+          <t>waveform_0020.00_post_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.027</v>
+        <v>0.07262299999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>0.027</v>
+        <v>0.07262</v>
       </c>
       <c r="F5">
         <f>(D5/E5-1)*100</f>
@@ -4750,19 +4756,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>waveform_0020.05_post_itsc_4turn.csv</t>
+          <t>waveform_0020.00_pre_healthy.csv</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>itsc_4turn</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.07262299999999999</v>
+        <v>0.027</v>
       </c>
       <c r="E6" t="n">
-        <v>0.07262</v>
+        <v>0.027</v>
       </c>
       <c r="F6">
         <f>(D6/E6-1)*100</f>
@@ -4781,19 +4787,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>waveform_0020.05_pre_healthy.csv</t>
+          <t>waveform_0020.04_post_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.027</v>
+        <v>0.07262299999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>0.027</v>
+        <v>0.07262</v>
       </c>
       <c r="F7">
         <f>(D7/E7-1)*100</f>
@@ -4812,19 +4818,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>waveform_0045.02_post_itsc_12turn.csv</t>
+          <t>waveform_0020.04_pre_healthy.csv</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>itsc_12turn</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.269578</v>
+        <v>0.027</v>
       </c>
       <c r="E8" t="n">
-        <v>0.26958</v>
+        <v>0.027</v>
       </c>
       <c r="F8">
         <f>(D8/E8-1)*100</f>
@@ -4843,7 +4849,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>waveform_0045.02_pre_itsc_4turn.csv</t>
+          <t>waveform_0020.05_post_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -4874,19 +4880,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>waveform_0045.03_post_itsc_12turn.csv</t>
+          <t>waveform_0020.05_pre_healthy.csv</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>itsc_12turn</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.269578</v>
+        <v>0.027</v>
       </c>
       <c r="E10" t="n">
-        <v>0.26958</v>
+        <v>0.027</v>
       </c>
       <c r="F10">
         <f>(D10/E10-1)*100</f>
@@ -4905,19 +4911,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>waveform_0045.03_pre_itsc_4turn.csv</t>
+          <t>waveform_0045.02_post_itsc_12turn.csv</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>itsc_4turn</t>
+          <t>itsc_12turn</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.07262299999999999</v>
+        <v>0.269578</v>
       </c>
       <c r="E11" t="n">
-        <v>0.07262</v>
+        <v>0.26958</v>
       </c>
       <c r="F11">
         <f>(D11/E11-1)*100</f>
@@ -4936,19 +4942,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>waveform_0075.04_post_overload.csv</t>
+          <t>waveform_0045.02_pre_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>overload</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.027</v>
+        <v>0.07262299999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>0.027</v>
+        <v>0.07262</v>
       </c>
       <c r="F12">
         <f>(D12/E12-1)*100</f>
@@ -4967,7 +4973,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>waveform_0075.04_pre_itsc_12turn.csv</t>
+          <t>waveform_0045.03_post_itsc_12turn.csv</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4998,19 +5004,19 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>waveform_0075.06_post_overload.csv</t>
+          <t>waveform_0045.03_pre_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>overload</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.027</v>
+        <v>0.07262299999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>0.027</v>
+        <v>0.07262</v>
       </c>
       <c r="F14">
         <f>(D14/E14-1)*100</f>
@@ -5029,19 +5035,19 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>waveform_0075.06_pre_itsc_12turn.csv</t>
+          <t>waveform_0075.04_post_overload.csv</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>itsc_12turn</t>
+          <t>overload</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.269578</v>
+        <v>0.027</v>
       </c>
       <c r="E15" t="n">
-        <v>0.26958</v>
+        <v>0.027</v>
       </c>
       <c r="F15">
         <f>(D15/E15-1)*100</f>
@@ -5060,19 +5066,19 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>waveform_0095.00_post_voltage_unbalance.csv</t>
+          <t>waveform_0075.04_pre_itsc_12turn.csv</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>voltage_unbalance</t>
+          <t>itsc_12turn</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.059508</v>
+        <v>0.269578</v>
       </c>
       <c r="E16" t="n">
-        <v>0.05951</v>
+        <v>0.26958</v>
       </c>
       <c r="F16">
         <f>(D16/E16-1)*100</f>
@@ -5091,7 +5097,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>waveform_0095.00_pre_overload.csv</t>
+          <t>waveform_0075.06_post_overload.csv</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5122,19 +5128,19 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>waveform_0095.01_post_voltage_unbalance.csv</t>
+          <t>waveform_0075.06_pre_itsc_12turn.csv</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>voltage_unbalance</t>
+          <t>itsc_12turn</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.059508</v>
+        <v>0.269578</v>
       </c>
       <c r="E18" t="n">
-        <v>0.05951</v>
+        <v>0.26958</v>
       </c>
       <c r="F18">
         <f>(D18/E18-1)*100</f>
@@ -5153,19 +5159,19 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>waveform_0095.01_pre_overload.csv</t>
+          <t>waveform_0095.00_post_voltage_unbalance.csv</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>overload</t>
+          <t>voltage_unbalance</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.027</v>
+        <v>0.059508</v>
       </c>
       <c r="E19" t="n">
-        <v>0.027</v>
+        <v>0.05951</v>
       </c>
       <c r="F19">
         <f>(D19/E19-1)*100</f>
@@ -5184,19 +5190,19 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>waveform_0120.02_post_single_phasing.csv</t>
+          <t>waveform_0095.00_pre_overload.csv</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>single_phasing</t>
+          <t>overload</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.479167</v>
+        <v>0.027</v>
       </c>
       <c r="E20" t="n">
-        <v>0.47917</v>
+        <v>0.027</v>
       </c>
       <c r="F20">
         <f>(D20/E20-1)*100</f>
@@ -5215,7 +5221,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>waveform_0120.02_pre_voltage_unbalance.csv</t>
+          <t>waveform_0095.01_post_voltage_unbalance.csv</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5246,12 +5252,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>waveform_0145.01_post_no_load.csv</t>
+          <t>waveform_0095.01_pre_overload.csv</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>no_load</t>
+          <t>overload</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -5277,19 +5283,19 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>waveform_0145.01_pre_single_phasing.csv</t>
+          <t>waveform_0095.04_post_voltage_unbalance.csv</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>single_phasing</t>
+          <t>voltage_unbalance</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.479167</v>
+        <v>0.059508</v>
       </c>
       <c r="E23" t="n">
-        <v>0.47917</v>
+        <v>0.05951</v>
       </c>
       <c r="F23">
         <f>(D23/E23-1)*100</f>
@@ -5308,12 +5314,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>waveform_0145.03_post_no_load.csv</t>
+          <t>waveform_0095.04_pre_overload.csv</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>no_load</t>
+          <t>overload</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -5339,7 +5345,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>waveform_0145.03_pre_single_phasing.csv</t>
+          <t>waveform_0120.02_post_single_phasing.csv</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -5370,19 +5376,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>waveform_0165.04_post_itsc_8turn.csv</t>
+          <t>waveform_0120.02_pre_voltage_unbalance.csv</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>itsc_8turn</t>
+          <t>voltage_unbalance</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.167573</v>
+        <v>0.059508</v>
       </c>
       <c r="E26" t="n">
-        <v>0.16757</v>
+        <v>0.05951</v>
       </c>
       <c r="F26">
         <f>(D26/E26-1)*100</f>
@@ -5401,19 +5407,19 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>waveform_0165.04_pre_no_load.csv</t>
+          <t>waveform_0120.06_post_single_phasing.csv</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>no_load</t>
+          <t>single_phasing</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.027</v>
+        <v>0.479167</v>
       </c>
       <c r="E27" t="n">
-        <v>0.027</v>
+        <v>0.47917</v>
       </c>
       <c r="F27">
         <f>(D27/E27-1)*100</f>
@@ -5432,19 +5438,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>waveform_0165.05_post_itsc_8turn.csv</t>
+          <t>waveform_0120.06_pre_voltage_unbalance.csv</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>itsc_8turn</t>
+          <t>voltage_unbalance</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.167573</v>
+        <v>0.059508</v>
       </c>
       <c r="E28" t="n">
-        <v>0.16757</v>
+        <v>0.05951</v>
       </c>
       <c r="F28">
         <f>(D28/E28-1)*100</f>
@@ -5463,7 +5469,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>waveform_0165.05_pre_no_load.csv</t>
+          <t>waveform_0145.00_post_no_load.csv</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -5494,19 +5500,19 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>waveform_0185.02_post_itsc_16turn.csv</t>
+          <t>waveform_0145.00_pre_single_phasing.csv</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>itsc_16turn</t>
+          <t>single_phasing</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.362533</v>
+        <v>0.479167</v>
       </c>
       <c r="E30" t="n">
-        <v>0.36253</v>
+        <v>0.47917</v>
       </c>
       <c r="F30">
         <f>(D30/E30-1)*100</f>
@@ -5525,19 +5531,19 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>waveform_0185.02_pre_itsc_8turn.csv</t>
+          <t>waveform_0145.01_post_no_load.csv</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>itsc_8turn</t>
+          <t>no_load</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.167573</v>
+        <v>0.027</v>
       </c>
       <c r="E31" t="n">
-        <v>0.16757</v>
+        <v>0.027</v>
       </c>
       <c r="F31">
         <f>(D31/E31-1)*100</f>
@@ -5556,19 +5562,19 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>waveform_0205.00_post_itsc_4turn_resistive.csv</t>
+          <t>waveform_0145.01_pre_single_phasing.csv</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>single_phasing</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.032438</v>
+        <v>0.479167</v>
       </c>
       <c r="E32" t="n">
-        <v>0.03244</v>
+        <v>0.47917</v>
       </c>
       <c r="F32">
         <f>(D32/E32-1)*100</f>
@@ -5587,19 +5593,19 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>waveform_0205.00_pre_itsc_16turn.csv</t>
+          <t>waveform_0145.03_post_no_load.csv</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>itsc_16turn</t>
+          <t>no_load</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.362533</v>
+        <v>0.027</v>
       </c>
       <c r="E33" t="n">
-        <v>0.36253</v>
+        <v>0.027</v>
       </c>
       <c r="F33">
         <f>(D33/E33-1)*100</f>
@@ -5618,19 +5624,19 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>waveform_0205.06_post_itsc_4turn_resistive.csv</t>
+          <t>waveform_0145.03_pre_single_phasing.csv</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>single_phasing</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.032438</v>
+        <v>0.479167</v>
       </c>
       <c r="E34" t="n">
-        <v>0.03244</v>
+        <v>0.47917</v>
       </c>
       <c r="F34">
         <f>(D34/E34-1)*100</f>
@@ -5649,19 +5655,19 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>waveform_0205.06_pre_itsc_16turn.csv</t>
+          <t>waveform_0165.03_post_itsc_8turn.csv</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>itsc_16turn</t>
+          <t>itsc_8turn</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.362533</v>
+        <v>0.167573</v>
       </c>
       <c r="E35" t="n">
-        <v>0.36253</v>
+        <v>0.16757</v>
       </c>
       <c r="F35">
         <f>(D35/E35-1)*100</f>
@@ -5680,19 +5686,19 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>waveform_0225.02_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0165.03_pre_no_load.csv</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>no_load</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.095294</v>
+        <v>0.027</v>
       </c>
       <c r="E36" t="n">
-        <v>0.09529</v>
+        <v>0.027</v>
       </c>
       <c r="F36">
         <f>(D36/E36-1)*100</f>
@@ -5711,19 +5717,19 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>waveform_0225.02_pre_itsc_4turn_resistive.csv</t>
+          <t>waveform_0165.04_post_itsc_8turn.csv</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>itsc_8turn</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.032438</v>
+        <v>0.167573</v>
       </c>
       <c r="E37" t="n">
-        <v>0.03244</v>
+        <v>0.16757</v>
       </c>
       <c r="F37">
         <f>(D37/E37-1)*100</f>
@@ -5742,19 +5748,19 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>waveform_0225.03_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0165.04_pre_no_load.csv</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>no_load</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.095294</v>
+        <v>0.027</v>
       </c>
       <c r="E38" t="n">
-        <v>0.09529</v>
+        <v>0.027</v>
       </c>
       <c r="F38">
         <f>(D38/E38-1)*100</f>
@@ -5773,19 +5779,19 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>waveform_0225.03_pre_itsc_4turn_resistive.csv</t>
+          <t>waveform_0165.05_post_itsc_8turn.csv</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>itsc_8turn</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.032438</v>
+        <v>0.167573</v>
       </c>
       <c r="E39" t="n">
-        <v>0.03244</v>
+        <v>0.16757</v>
       </c>
       <c r="F39">
         <f>(D39/E39-1)*100</f>
@@ -5804,19 +5810,19 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>waveform_0245.02_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0165.05_pre_no_load.csv</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>no_load</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.095294</v>
+        <v>0.027</v>
       </c>
       <c r="E40" t="n">
-        <v>0.09529</v>
+        <v>0.027</v>
       </c>
       <c r="F40">
         <f>(D40/E40-1)*100</f>
@@ -5835,19 +5841,19 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>waveform_0245.02_pre_itsc_4turn_halfload.csv</t>
+          <t>waveform_0185.02_post_itsc_16turn.csv</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>itsc_16turn</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.095294</v>
+        <v>0.362533</v>
       </c>
       <c r="E41" t="n">
-        <v>0.09529</v>
+        <v>0.36253</v>
       </c>
       <c r="F41">
         <f>(D41/E41-1)*100</f>
@@ -5866,19 +5872,19 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>waveform_0245.04_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0185.02_pre_itsc_8turn.csv</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>itsc_8turn</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.095294</v>
+        <v>0.167573</v>
       </c>
       <c r="E42" t="n">
-        <v>0.09529</v>
+        <v>0.16757</v>
       </c>
       <c r="F42">
         <f>(D42/E42-1)*100</f>
@@ -5897,19 +5903,19 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>waveform_0245.04_pre_itsc_4turn_halfload.csv</t>
+          <t>waveform_0205.00_post_itsc_4turn_resistive.csv</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>itsc_4turn_resistive</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.095294</v>
+        <v>0.032438</v>
       </c>
       <c r="E43" t="n">
-        <v>0.09529</v>
+        <v>0.03244</v>
       </c>
       <c r="F43">
         <f>(D43/E43-1)*100</f>
@@ -5923,24 +5929,24 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>waveform_0000.00_post_healthy.csv</t>
+          <t>waveform_0205.00_pre_itsc_16turn.csv</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>itsc_16turn</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.027</v>
+        <v>0.362533</v>
       </c>
       <c r="E44" t="n">
-        <v>0.027</v>
+        <v>0.36253</v>
       </c>
       <c r="F44">
         <f>(D44/E44-1)*100</f>
@@ -5954,24 +5960,24 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>waveform_0000.01_post_healthy.csv</t>
+          <t>waveform_0205.05_post_itsc_4turn_resistive.csv</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>itsc_4turn_resistive</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.027</v>
+        <v>0.032438</v>
       </c>
       <c r="E45" t="n">
-        <v>0.027</v>
+        <v>0.03244</v>
       </c>
       <c r="F45">
         <f>(D45/E45-1)*100</f>
@@ -5985,24 +5991,24 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>waveform_0020.04_post_itsc_4turn.csv</t>
+          <t>waveform_0205.05_pre_itsc_16turn.csv</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>itsc_4turn</t>
+          <t>itsc_16turn</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.06833699999999999</v>
+        <v>0.362533</v>
       </c>
       <c r="E46" t="n">
-        <v>0.06834</v>
+        <v>0.36253</v>
       </c>
       <c r="F46">
         <f>(D46/E46-1)*100</f>
@@ -6016,24 +6022,24 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>waveform_0020.04_pre_healthy.csv</t>
+          <t>waveform_0205.06_post_itsc_4turn_resistive.csv</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>itsc_4turn_resistive</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.027</v>
+        <v>0.032438</v>
       </c>
       <c r="E47" t="n">
-        <v>0.027</v>
+        <v>0.03244</v>
       </c>
       <c r="F47">
         <f>(D47/E47-1)*100</f>
@@ -6047,24 +6053,24 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>waveform_0020.06_post_itsc_4turn.csv</t>
+          <t>waveform_0205.06_pre_itsc_16turn.csv</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>itsc_4turn</t>
+          <t>itsc_16turn</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.06833699999999999</v>
+        <v>0.362533</v>
       </c>
       <c r="E48" t="n">
-        <v>0.06834</v>
+        <v>0.36253</v>
       </c>
       <c r="F48">
         <f>(D48/E48-1)*100</f>
@@ -6078,24 +6084,24 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>waveform_0020.06_pre_healthy.csv</t>
+          <t>waveform_0225.01_post_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.027</v>
+        <v>0.095294</v>
       </c>
       <c r="E49" t="n">
-        <v>0.027</v>
+        <v>0.09529</v>
       </c>
       <c r="F49">
         <f>(D49/E49-1)*100</f>
@@ -6109,24 +6115,24 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>waveform_0045.01_post_itsc_12turn.csv</t>
+          <t>waveform_0225.01_pre_itsc_4turn_resistive.csv</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>itsc_12turn</t>
+          <t>itsc_4turn_resistive</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.259428</v>
+        <v>0.032438</v>
       </c>
       <c r="E50" t="n">
-        <v>0.25943</v>
+        <v>0.03244</v>
       </c>
       <c r="F50">
         <f>(D50/E50-1)*100</f>
@@ -6140,24 +6146,24 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>waveform_0045.01_pre_itsc_4turn.csv</t>
+          <t>waveform_0225.02_post_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>itsc_4turn</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.06833699999999999</v>
+        <v>0.095294</v>
       </c>
       <c r="E51" t="n">
-        <v>0.06834</v>
+        <v>0.09529</v>
       </c>
       <c r="F51">
         <f>(D51/E51-1)*100</f>
@@ -6171,24 +6177,24 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>waveform_0045.04_post_itsc_12turn.csv</t>
+          <t>waveform_0225.02_pre_itsc_4turn_resistive.csv</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>itsc_12turn</t>
+          <t>itsc_4turn_resistive</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.259428</v>
+        <v>0.032438</v>
       </c>
       <c r="E52" t="n">
-        <v>0.25943</v>
+        <v>0.03244</v>
       </c>
       <c r="F52">
         <f>(D52/E52-1)*100</f>
@@ -6202,24 +6208,24 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>waveform_0045.04_pre_itsc_4turn.csv</t>
+          <t>waveform_0225.03_post_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>itsc_4turn</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.06833699999999999</v>
+        <v>0.095294</v>
       </c>
       <c r="E53" t="n">
-        <v>0.06834</v>
+        <v>0.09529</v>
       </c>
       <c r="F53">
         <f>(D53/E53-1)*100</f>
@@ -6233,24 +6239,24 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>waveform_0075.01_post_overload.csv</t>
+          <t>waveform_0225.03_pre_itsc_4turn_resistive.csv</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>overload</t>
+          <t>itsc_4turn_resistive</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.027</v>
+        <v>0.032438</v>
       </c>
       <c r="E54" t="n">
-        <v>0.027</v>
+        <v>0.03244</v>
       </c>
       <c r="F54">
         <f>(D54/E54-1)*100</f>
@@ -6264,24 +6270,24 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>waveform_0075.01_pre_itsc_12turn.csv</t>
+          <t>waveform_0245.02_post_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>itsc_12turn</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.259428</v>
+        <v>0.095294</v>
       </c>
       <c r="E55" t="n">
-        <v>0.25943</v>
+        <v>0.09529</v>
       </c>
       <c r="F55">
         <f>(D55/E55-1)*100</f>
@@ -6295,24 +6301,24 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>waveform_0075.05_post_overload.csv</t>
+          <t>waveform_0245.02_pre_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>overload</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.027</v>
+        <v>0.095294</v>
       </c>
       <c r="E56" t="n">
-        <v>0.027</v>
+        <v>0.09529</v>
       </c>
       <c r="F56">
         <f>(D56/E56-1)*100</f>
@@ -6326,24 +6332,24 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>waveform_0075.05_pre_itsc_12turn.csv</t>
+          <t>waveform_0245.03_post_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>itsc_12turn</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.259428</v>
+        <v>0.095294</v>
       </c>
       <c r="E57" t="n">
-        <v>0.25943</v>
+        <v>0.09529</v>
       </c>
       <c r="F57">
         <f>(D57/E57-1)*100</f>
@@ -6357,24 +6363,24 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>waveform_0095.04_post_voltage_unbalance.csv</t>
+          <t>waveform_0245.03_pre_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>voltage_unbalance</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.059508</v>
+        <v>0.095294</v>
       </c>
       <c r="E58" t="n">
-        <v>0.05951</v>
+        <v>0.09529</v>
       </c>
       <c r="F58">
         <f>(D58/E58-1)*100</f>
@@ -6388,24 +6394,24 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>waveform_0095.04_pre_overload.csv</t>
+          <t>waveform_0245.04_post_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>overload</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.027</v>
+        <v>0.095294</v>
       </c>
       <c r="E59" t="n">
-        <v>0.027</v>
+        <v>0.09529</v>
       </c>
       <c r="F59">
         <f>(D59/E59-1)*100</f>
@@ -6419,24 +6425,24 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>a90</t>
+          <t>a0</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>waveform_0095.05_post_voltage_unbalance.csv</t>
+          <t>waveform_0245.04_pre_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>voltage_unbalance</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.059508</v>
+        <v>0.095294</v>
       </c>
       <c r="E60" t="n">
-        <v>0.05951</v>
+        <v>0.09529</v>
       </c>
       <c r="F60">
         <f>(D60/E60-1)*100</f>
@@ -6455,12 +6461,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>waveform_0095.05_pre_overload.csv</t>
+          <t>waveform_0000.00_post_healthy.csv</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>overload</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -6486,19 +6492,19 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>waveform_0120.01_post_single_phasing.csv</t>
+          <t>waveform_0000.01_post_healthy.csv</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>single_phasing</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.479167</v>
+        <v>0.027</v>
       </c>
       <c r="E62" t="n">
-        <v>0.47917</v>
+        <v>0.027</v>
       </c>
       <c r="F62">
         <f>(D62/E62-1)*100</f>
@@ -6517,19 +6523,19 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>waveform_0120.01_pre_voltage_unbalance.csv</t>
+          <t>waveform_0000.07_post_healthy.csv</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>voltage_unbalance</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.059508</v>
+        <v>0.027</v>
       </c>
       <c r="E63" t="n">
-        <v>0.05951</v>
+        <v>0.027</v>
       </c>
       <c r="F63">
         <f>(D63/E63-1)*100</f>
@@ -6548,19 +6554,19 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>waveform_0120.05_post_single_phasing.csv</t>
+          <t>waveform_0020.04_post_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>single_phasing</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.479167</v>
+        <v>0.06833699999999999</v>
       </c>
       <c r="E64" t="n">
-        <v>0.47917</v>
+        <v>0.06834</v>
       </c>
       <c r="F64">
         <f>(D64/E64-1)*100</f>
@@ -6579,19 +6585,19 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>waveform_0120.05_pre_voltage_unbalance.csv</t>
+          <t>waveform_0020.04_pre_healthy.csv</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>voltage_unbalance</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.059508</v>
+        <v>0.027</v>
       </c>
       <c r="E65" t="n">
-        <v>0.05951</v>
+        <v>0.027</v>
       </c>
       <c r="F65">
         <f>(D65/E65-1)*100</f>
@@ -6610,19 +6616,19 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>waveform_0145.00_post_no_load.csv</t>
+          <t>waveform_0020.06_post_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>no_load</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.027</v>
+        <v>0.06833699999999999</v>
       </c>
       <c r="E66" t="n">
-        <v>0.027</v>
+        <v>0.06834</v>
       </c>
       <c r="F66">
         <f>(D66/E66-1)*100</f>
@@ -6641,19 +6647,19 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>waveform_0145.00_pre_single_phasing.csv</t>
+          <t>waveform_0020.06_pre_healthy.csv</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>single_phasing</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.479167</v>
+        <v>0.027</v>
       </c>
       <c r="E67" t="n">
-        <v>0.47917</v>
+        <v>0.027</v>
       </c>
       <c r="F67">
         <f>(D67/E67-1)*100</f>
@@ -6672,19 +6678,19 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>waveform_0165.00_post_itsc_8turn.csv</t>
+          <t>waveform_0045.01_post_itsc_12turn.csv</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>itsc_8turn</t>
+          <t>itsc_12turn</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.160109</v>
+        <v>0.259428</v>
       </c>
       <c r="E68" t="n">
-        <v>0.16011</v>
+        <v>0.25943</v>
       </c>
       <c r="F68">
         <f>(D68/E68-1)*100</f>
@@ -6703,19 +6709,19 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>waveform_0165.00_pre_no_load.csv</t>
+          <t>waveform_0045.01_pre_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>no_load</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.027</v>
+        <v>0.06833699999999999</v>
       </c>
       <c r="E69" t="n">
-        <v>0.027</v>
+        <v>0.06834</v>
       </c>
       <c r="F69">
         <f>(D69/E69-1)*100</f>
@@ -6734,19 +6740,19 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>waveform_0165.03_post_itsc_8turn.csv</t>
+          <t>waveform_0045.04_post_itsc_12turn.csv</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>itsc_8turn</t>
+          <t>itsc_12turn</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.160109</v>
+        <v>0.259428</v>
       </c>
       <c r="E70" t="n">
-        <v>0.16011</v>
+        <v>0.25943</v>
       </c>
       <c r="F70">
         <f>(D70/E70-1)*100</f>
@@ -6765,19 +6771,19 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>waveform_0165.03_pre_no_load.csv</t>
+          <t>waveform_0045.04_pre_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>no_load</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.027</v>
+        <v>0.06833699999999999</v>
       </c>
       <c r="E71" t="n">
-        <v>0.027</v>
+        <v>0.06834</v>
       </c>
       <c r="F71">
         <f>(D71/E71-1)*100</f>
@@ -6796,19 +6802,19 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>waveform_0185.01_post_itsc_16turn.csv</t>
+          <t>waveform_0045.05_post_itsc_12turn.csv</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>itsc_16turn</t>
+          <t>itsc_12turn</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.350064</v>
+        <v>0.259428</v>
       </c>
       <c r="E72" t="n">
-        <v>0.35006</v>
+        <v>0.25943</v>
       </c>
       <c r="F72">
         <f>(D72/E72-1)*100</f>
@@ -6827,19 +6833,19 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>waveform_0185.01_pre_itsc_8turn.csv</t>
+          <t>waveform_0045.05_pre_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>itsc_8turn</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.160109</v>
+        <v>0.06833699999999999</v>
       </c>
       <c r="E73" t="n">
-        <v>0.16011</v>
+        <v>0.06834</v>
       </c>
       <c r="F73">
         <f>(D73/E73-1)*100</f>
@@ -6858,19 +6864,19 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>waveform_0185.03_post_itsc_16turn.csv</t>
+          <t>waveform_0075.01_post_overload.csv</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>itsc_16turn</t>
+          <t>overload</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.350064</v>
+        <v>0.027</v>
       </c>
       <c r="E74" t="n">
-        <v>0.35006</v>
+        <v>0.027</v>
       </c>
       <c r="F74">
         <f>(D74/E74-1)*100</f>
@@ -6889,19 +6895,19 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>waveform_0185.03_pre_itsc_8turn.csv</t>
+          <t>waveform_0075.01_pre_itsc_12turn.csv</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>itsc_8turn</t>
+          <t>itsc_12turn</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.160109</v>
+        <v>0.259428</v>
       </c>
       <c r="E75" t="n">
-        <v>0.16011</v>
+        <v>0.25943</v>
       </c>
       <c r="F75">
         <f>(D75/E75-1)*100</f>
@@ -6920,19 +6926,19 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>waveform_0205.05_post_itsc_4turn_resistive.csv</t>
+          <t>waveform_0075.03_post_overload.csv</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>overload</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.031407</v>
+        <v>0.027</v>
       </c>
       <c r="E76" t="n">
-        <v>0.03141</v>
+        <v>0.027</v>
       </c>
       <c r="F76">
         <f>(D76/E76-1)*100</f>
@@ -6951,19 +6957,19 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>waveform_0205.05_pre_itsc_16turn.csv</t>
+          <t>waveform_0075.03_pre_itsc_12turn.csv</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>itsc_16turn</t>
+          <t>itsc_12turn</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.350064</v>
+        <v>0.259428</v>
       </c>
       <c r="E77" t="n">
-        <v>0.35006</v>
+        <v>0.25943</v>
       </c>
       <c r="F77">
         <f>(D77/E77-1)*100</f>
@@ -6982,19 +6988,19 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>waveform_0205.06_post_itsc_4turn_resistive.csv</t>
+          <t>waveform_0075.05_post_overload.csv</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>overload</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0.031407</v>
+        <v>0.027</v>
       </c>
       <c r="E78" t="n">
-        <v>0.03141</v>
+        <v>0.027</v>
       </c>
       <c r="F78">
         <f>(D78/E78-1)*100</f>
@@ -7013,19 +7019,19 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>waveform_0205.06_pre_itsc_16turn.csv</t>
+          <t>waveform_0075.05_pre_itsc_12turn.csv</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>itsc_16turn</t>
+          <t>itsc_12turn</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.350064</v>
+        <v>0.259428</v>
       </c>
       <c r="E79" t="n">
-        <v>0.35006</v>
+        <v>0.25943</v>
       </c>
       <c r="F79">
         <f>(D79/E79-1)*100</f>
@@ -7044,19 +7050,19 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>waveform_0225.03_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0095.02_post_voltage_unbalance.csv</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>voltage_unbalance</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.09618</v>
+        <v>0.059508</v>
       </c>
       <c r="E80" t="n">
-        <v>0.09618</v>
+        <v>0.05951</v>
       </c>
       <c r="F80">
         <f>(D80/E80-1)*100</f>
@@ -7075,19 +7081,19 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>waveform_0225.03_pre_itsc_4turn_resistive.csv</t>
+          <t>waveform_0095.02_pre_overload.csv</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>overload</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.031407</v>
+        <v>0.027</v>
       </c>
       <c r="E81" t="n">
-        <v>0.03141</v>
+        <v>0.027</v>
       </c>
       <c r="F81">
         <f>(D81/E81-1)*100</f>
@@ -7106,19 +7112,19 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>waveform_0225.05_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0095.04_post_voltage_unbalance.csv</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>voltage_unbalance</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.09618</v>
+        <v>0.059508</v>
       </c>
       <c r="E82" t="n">
-        <v>0.09618</v>
+        <v>0.05951</v>
       </c>
       <c r="F82">
         <f>(D82/E82-1)*100</f>
@@ -7137,19 +7143,19 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>waveform_0225.05_pre_itsc_4turn_resistive.csv</t>
+          <t>waveform_0095.04_pre_overload.csv</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>overload</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0.031407</v>
+        <v>0.027</v>
       </c>
       <c r="E83" t="n">
-        <v>0.03141</v>
+        <v>0.027</v>
       </c>
       <c r="F83">
         <f>(D83/E83-1)*100</f>
@@ -7168,19 +7174,19 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>waveform_0245.03_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0095.05_post_voltage_unbalance.csv</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>voltage_unbalance</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0.09618</v>
+        <v>0.059508</v>
       </c>
       <c r="E84" t="n">
-        <v>0.09618</v>
+        <v>0.05951</v>
       </c>
       <c r="F84">
         <f>(D84/E84-1)*100</f>
@@ -7199,19 +7205,19 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>waveform_0245.03_pre_itsc_4turn_halfload.csv</t>
+          <t>waveform_0095.05_pre_overload.csv</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>overload</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>0.09618</v>
+        <v>0.027</v>
       </c>
       <c r="E85" t="n">
-        <v>0.09618</v>
+        <v>0.027</v>
       </c>
       <c r="F85">
         <f>(D85/E85-1)*100</f>
@@ -7230,19 +7236,19 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>waveform_0245.05_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0120.01_post_single_phasing.csv</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>single_phasing</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.09618</v>
+        <v>0.479167</v>
       </c>
       <c r="E86" t="n">
-        <v>0.09618</v>
+        <v>0.47917</v>
       </c>
       <c r="F86">
         <f>(D86/E86-1)*100</f>
@@ -7261,19 +7267,19 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>waveform_0245.05_pre_itsc_4turn_halfload.csv</t>
+          <t>waveform_0120.01_pre_voltage_unbalance.csv</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>voltage_unbalance</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.09618</v>
+        <v>0.059508</v>
       </c>
       <c r="E87" t="n">
-        <v>0.09618</v>
+        <v>0.05951</v>
       </c>
       <c r="F87">
         <f>(D87/E87-1)*100</f>
@@ -7287,24 +7293,24 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>waveform_0000.00_post_healthy.csv</t>
+          <t>waveform_0120.05_post_single_phasing.csv</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>single_phasing</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.027</v>
+        <v>0.479167</v>
       </c>
       <c r="E88" t="n">
-        <v>0.027</v>
+        <v>0.47917</v>
       </c>
       <c r="F88">
         <f>(D88/E88-1)*100</f>
@@ -7318,24 +7324,24 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>waveform_0020.00_post_itsc_4turn.csv</t>
+          <t>waveform_0120.05_pre_voltage_unbalance.csv</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>itsc_4turn</t>
+          <t>voltage_unbalance</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.031298</v>
+        <v>0.059508</v>
       </c>
       <c r="E89" t="n">
-        <v>0.0313</v>
+        <v>0.05951</v>
       </c>
       <c r="F89">
         <f>(D89/E89-1)*100</f>
@@ -7349,17 +7355,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>waveform_0020.00_pre_healthy.csv</t>
+          <t>waveform_0145.00_post_no_load.csv</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>no_load</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -7380,24 +7386,24 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>waveform_0020.03_post_itsc_4turn.csv</t>
+          <t>waveform_0145.00_pre_single_phasing.csv</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>itsc_4turn</t>
+          <t>single_phasing</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.031298</v>
+        <v>0.479167</v>
       </c>
       <c r="E91" t="n">
-        <v>0.0313</v>
+        <v>0.47917</v>
       </c>
       <c r="F91">
         <f>(D91/E91-1)*100</f>
@@ -7411,17 +7417,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>waveform_0020.03_pre_healthy.csv</t>
+          <t>waveform_0145.03_post_no_load.csv</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>no_load</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -7442,24 +7448,24 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>waveform_0045.02_post_itsc_12turn.csv</t>
+          <t>waveform_0145.03_pre_single_phasing.csv</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>itsc_12turn</t>
+          <t>single_phasing</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0.222124</v>
+        <v>0.479167</v>
       </c>
       <c r="E93" t="n">
-        <v>0.22212</v>
+        <v>0.47917</v>
       </c>
       <c r="F93">
         <f>(D93/E93-1)*100</f>
@@ -7473,24 +7479,24 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>waveform_0045.02_pre_itsc_4turn.csv</t>
+          <t>waveform_0165.00_post_itsc_8turn.csv</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>itsc_4turn</t>
+          <t>itsc_8turn</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.031298</v>
+        <v>0.160109</v>
       </c>
       <c r="E94" t="n">
-        <v>0.0313</v>
+        <v>0.16011</v>
       </c>
       <c r="F94">
         <f>(D94/E94-1)*100</f>
@@ -7504,17 +7510,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>waveform_0075.02_post_overload.csv</t>
+          <t>waveform_0165.00_pre_no_load.csv</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>overload</t>
+          <t>no_load</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -7535,24 +7541,24 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>waveform_0075.02_pre_itsc_12turn.csv</t>
+          <t>waveform_0165.03_post_itsc_8turn.csv</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>itsc_12turn</t>
+          <t>itsc_8turn</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0.222124</v>
+        <v>0.160109</v>
       </c>
       <c r="E96" t="n">
-        <v>0.22212</v>
+        <v>0.16011</v>
       </c>
       <c r="F96">
         <f>(D96/E96-1)*100</f>
@@ -7566,17 +7572,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>waveform_0075.05_post_overload.csv</t>
+          <t>waveform_0165.03_pre_no_load.csv</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>overload</t>
+          <t>no_load</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -7597,24 +7603,24 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>waveform_0075.05_pre_itsc_12turn.csv</t>
+          <t>waveform_0165.08_post_itsc_8turn.csv</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>itsc_12turn</t>
+          <t>itsc_8turn</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0.222124</v>
+        <v>0.160109</v>
       </c>
       <c r="E98" t="n">
-        <v>0.22212</v>
+        <v>0.16011</v>
       </c>
       <c r="F98">
         <f>(D98/E98-1)*100</f>
@@ -7628,24 +7634,24 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>waveform_0095.02_post_voltage_unbalance.csv</t>
+          <t>waveform_0165.08_pre_no_load.csv</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>voltage_unbalance</t>
+          <t>no_load</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0.059508</v>
+        <v>0.027</v>
       </c>
       <c r="E99" t="n">
-        <v>0.05951</v>
+        <v>0.027</v>
       </c>
       <c r="F99">
         <f>(D99/E99-1)*100</f>
@@ -7659,24 +7665,24 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>waveform_0095.02_pre_overload.csv</t>
+          <t>waveform_0185.01_post_itsc_16turn.csv</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>overload</t>
+          <t>itsc_16turn</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0.027</v>
+        <v>0.350064</v>
       </c>
       <c r="E100" t="n">
-        <v>0.027</v>
+        <v>0.35006</v>
       </c>
       <c r="F100">
         <f>(D100/E100-1)*100</f>
@@ -7690,24 +7696,24 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>waveform_0120.04_post_single_phasing.csv</t>
+          <t>waveform_0185.01_pre_itsc_8turn.csv</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>single_phasing</t>
+          <t>itsc_8turn</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.479167</v>
+        <v>0.160109</v>
       </c>
       <c r="E101" t="n">
-        <v>0.47917</v>
+        <v>0.16011</v>
       </c>
       <c r="F101">
         <f>(D101/E101-1)*100</f>
@@ -7721,24 +7727,24 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>waveform_0120.04_pre_voltage_unbalance.csv</t>
+          <t>waveform_0185.03_post_itsc_16turn.csv</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>voltage_unbalance</t>
+          <t>itsc_16turn</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.059508</v>
+        <v>0.350064</v>
       </c>
       <c r="E102" t="n">
-        <v>0.05951</v>
+        <v>0.35006</v>
       </c>
       <c r="F102">
         <f>(D102/E102-1)*100</f>
@@ -7752,24 +7758,24 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>waveform_0120.05_post_single_phasing.csv</t>
+          <t>waveform_0185.03_pre_itsc_8turn.csv</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>single_phasing</t>
+          <t>itsc_8turn</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.479167</v>
+        <v>0.160109</v>
       </c>
       <c r="E103" t="n">
-        <v>0.47917</v>
+        <v>0.16011</v>
       </c>
       <c r="F103">
         <f>(D103/E103-1)*100</f>
@@ -7783,24 +7789,24 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>waveform_0120.05_pre_voltage_unbalance.csv</t>
+          <t>waveform_0205.03_post_itsc_4turn_resistive.csv</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>voltage_unbalance</t>
+          <t>itsc_4turn_resistive</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.059508</v>
+        <v>0.031407</v>
       </c>
       <c r="E104" t="n">
-        <v>0.05951</v>
+        <v>0.03141</v>
       </c>
       <c r="F104">
         <f>(D104/E104-1)*100</f>
@@ -7814,24 +7820,24 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>waveform_0145.05_post_no_load.csv</t>
+          <t>waveform_0205.03_pre_itsc_16turn.csv</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>no_load</t>
+          <t>itsc_16turn</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.027</v>
+        <v>0.350064</v>
       </c>
       <c r="E105" t="n">
-        <v>0.027</v>
+        <v>0.35006</v>
       </c>
       <c r="F105">
         <f>(D105/E105-1)*100</f>
@@ -7845,24 +7851,24 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>waveform_0145.05_pre_single_phasing.csv</t>
+          <t>waveform_0205.05_post_itsc_4turn_resistive.csv</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>single_phasing</t>
+          <t>itsc_4turn_resistive</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.479167</v>
+        <v>0.031407</v>
       </c>
       <c r="E106" t="n">
-        <v>0.47917</v>
+        <v>0.03141</v>
       </c>
       <c r="F106">
         <f>(D106/E106-1)*100</f>
@@ -7876,24 +7882,24 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>waveform_0145.06_post_no_load.csv</t>
+          <t>waveform_0205.05_pre_itsc_16turn.csv</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>no_load</t>
+          <t>itsc_16turn</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.027</v>
+        <v>0.350064</v>
       </c>
       <c r="E107" t="n">
-        <v>0.027</v>
+        <v>0.35006</v>
       </c>
       <c r="F107">
         <f>(D107/E107-1)*100</f>
@@ -7907,24 +7913,24 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>waveform_0145.06_pre_single_phasing.csv</t>
+          <t>waveform_0205.06_post_itsc_4turn_resistive.csv</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>single_phasing</t>
+          <t>itsc_4turn_resistive</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0.479167</v>
+        <v>0.031407</v>
       </c>
       <c r="E108" t="n">
-        <v>0.47917</v>
+        <v>0.03141</v>
       </c>
       <c r="F108">
         <f>(D108/E108-1)*100</f>
@@ -7938,24 +7944,24 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>waveform_0165.04_post_itsc_8turn.csv</t>
+          <t>waveform_0205.06_pre_itsc_16turn.csv</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>itsc_8turn</t>
+          <t>itsc_16turn</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.122089</v>
+        <v>0.350064</v>
       </c>
       <c r="E109" t="n">
-        <v>0.12209</v>
+        <v>0.35006</v>
       </c>
       <c r="F109">
         <f>(D109/E109-1)*100</f>
@@ -7969,24 +7975,24 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>waveform_0165.04_pre_no_load.csv</t>
+          <t>waveform_0225.03_post_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>no_load</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.027</v>
+        <v>0.09618</v>
       </c>
       <c r="E110" t="n">
-        <v>0.027</v>
+        <v>0.09618</v>
       </c>
       <c r="F110">
         <f>(D110/E110-1)*100</f>
@@ -8000,24 +8006,24 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>waveform_0165.06_post_itsc_8turn.csv</t>
+          <t>waveform_0225.03_pre_itsc_4turn_resistive.csv</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>itsc_8turn</t>
+          <t>itsc_4turn_resistive</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.122089</v>
+        <v>0.031407</v>
       </c>
       <c r="E111" t="n">
-        <v>0.12209</v>
+        <v>0.03141</v>
       </c>
       <c r="F111">
         <f>(D111/E111-1)*100</f>
@@ -8031,24 +8037,24 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>waveform_0165.06_pre_no_load.csv</t>
+          <t>waveform_0225.05_post_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>no_load</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.027</v>
+        <v>0.09618</v>
       </c>
       <c r="E112" t="n">
-        <v>0.027</v>
+        <v>0.09618</v>
       </c>
       <c r="F112">
         <f>(D112/E112-1)*100</f>
@@ -8062,24 +8068,24 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>waveform_0185.03_post_itsc_16turn.csv</t>
+          <t>waveform_0225.05_pre_itsc_4turn_resistive.csv</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>itsc_16turn</t>
+          <t>itsc_4turn_resistive</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.313563</v>
+        <v>0.031407</v>
       </c>
       <c r="E113" t="n">
-        <v>0.31356</v>
+        <v>0.03141</v>
       </c>
       <c r="F113">
         <f>(D113/E113-1)*100</f>
@@ -8093,24 +8099,24 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>waveform_0185.03_pre_itsc_8turn.csv</t>
+          <t>waveform_0245.03_post_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>itsc_8turn</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.122089</v>
+        <v>0.09618</v>
       </c>
       <c r="E114" t="n">
-        <v>0.12209</v>
+        <v>0.09618</v>
       </c>
       <c r="F114">
         <f>(D114/E114-1)*100</f>
@@ -8124,24 +8130,24 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>waveform_0185.05_post_itsc_16turn.csv</t>
+          <t>waveform_0245.03_pre_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>itsc_16turn</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0.313563</v>
+        <v>0.09618</v>
       </c>
       <c r="E115" t="n">
-        <v>0.31356</v>
+        <v>0.09618</v>
       </c>
       <c r="F115">
         <f>(D115/E115-1)*100</f>
@@ -8155,24 +8161,24 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>waveform_0185.05_pre_itsc_8turn.csv</t>
+          <t>waveform_0245.05_post_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>itsc_8turn</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>0.122089</v>
+        <v>0.09618</v>
       </c>
       <c r="E116" t="n">
-        <v>0.12209</v>
+        <v>0.09618</v>
       </c>
       <c r="F116">
         <f>(D116/E116-1)*100</f>
@@ -8186,24 +8192,24 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>waveform_0205.00_post_itsc_4turn_resistive.csv</t>
+          <t>waveform_0245.05_pre_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>0.022165</v>
+        <v>0.09618</v>
       </c>
       <c r="E117" t="n">
-        <v>0.02217</v>
+        <v>0.09618</v>
       </c>
       <c r="F117">
         <f>(D117/E117-1)*100</f>
@@ -8217,24 +8223,24 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>waveform_0205.00_pre_itsc_16turn.csv</t>
+          <t>waveform_0245.07_post_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>itsc_16turn</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0.313563</v>
+        <v>0.09618</v>
       </c>
       <c r="E118" t="n">
-        <v>0.31356</v>
+        <v>0.09618</v>
       </c>
       <c r="F118">
         <f>(D118/E118-1)*100</f>
@@ -8248,24 +8254,24 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>a180</t>
+          <t>a90</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>waveform_0205.04_post_itsc_4turn_resistive.csv</t>
+          <t>waveform_0245.07_pre_itsc_4turn_halfload.csv</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>itsc_4turn_halfload</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>0.022165</v>
+        <v>0.09618</v>
       </c>
       <c r="E119" t="n">
-        <v>0.02217</v>
+        <v>0.09618</v>
       </c>
       <c r="F119">
         <f>(D119/E119-1)*100</f>
@@ -8284,19 +8290,19 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>waveform_0205.04_pre_itsc_16turn.csv</t>
+          <t>waveform_0000.00_post_healthy.csv</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>itsc_16turn</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>0.313563</v>
+        <v>0.027</v>
       </c>
       <c r="E120" t="n">
-        <v>0.31356</v>
+        <v>0.027</v>
       </c>
       <c r="F120">
         <f>(D120/E120-1)*100</f>
@@ -8315,19 +8321,19 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>waveform_0225.02_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0000.08_post_healthy.csv</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>0.05955</v>
+        <v>0.027</v>
       </c>
       <c r="E121" t="n">
-        <v>0.05955</v>
+        <v>0.027</v>
       </c>
       <c r="F121">
         <f>(D121/E121-1)*100</f>
@@ -8346,19 +8352,19 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>waveform_0225.02_pre_itsc_4turn_resistive.csv</t>
+          <t>waveform_0020.00_post_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>0.022165</v>
+        <v>0.031298</v>
       </c>
       <c r="E122" t="n">
-        <v>0.02217</v>
+        <v>0.0313</v>
       </c>
       <c r="F122">
         <f>(D122/E122-1)*100</f>
@@ -8377,19 +8383,19 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>waveform_0225.03_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0020.00_pre_healthy.csv</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>0.059549</v>
+        <v>0.027</v>
       </c>
       <c r="E123" t="n">
-        <v>0.05955</v>
+        <v>0.027</v>
       </c>
       <c r="F123">
         <f>(D123/E123-1)*100</f>
@@ -8408,19 +8414,19 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>waveform_0225.03_pre_itsc_4turn_resistive.csv</t>
+          <t>waveform_0020.02_post_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>itsc_4turn_resistive</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>0.022165</v>
+        <v>0.031298</v>
       </c>
       <c r="E124" t="n">
-        <v>0.02217</v>
+        <v>0.0313</v>
       </c>
       <c r="F124">
         <f>(D124/E124-1)*100</f>
@@ -8439,19 +8445,19 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>waveform_0245.02_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0020.02_pre_healthy.csv</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>0.05955</v>
+        <v>0.027</v>
       </c>
       <c r="E125" t="n">
-        <v>0.05955</v>
+        <v>0.027</v>
       </c>
       <c r="F125">
         <f>(D125/E125-1)*100</f>
@@ -8470,19 +8476,19 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>waveform_0245.02_pre_itsc_4turn_halfload.csv</t>
+          <t>waveform_0020.03_post_itsc_4turn.csv</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>itsc_4turn</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>0.05955</v>
+        <v>0.031298</v>
       </c>
       <c r="E126" t="n">
-        <v>0.05955</v>
+        <v>0.0313</v>
       </c>
       <c r="F126">
         <f>(D126/E126-1)*100</f>
@@ -8501,19 +8507,19 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>waveform_0245.04_post_itsc_4turn_halfload.csv</t>
+          <t>waveform_0020.03_pre_healthy.csv</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>healthy</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>0.059549</v>
+        <v>0.027</v>
       </c>
       <c r="E127" t="n">
-        <v>0.05955</v>
+        <v>0.027</v>
       </c>
       <c r="F127">
         <f>(D127/E127-1)*100</f>
@@ -8532,19 +8538,19 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>waveform_0245.04_pre_itsc_4turn_halfload.csv</t>
+          <t>waveform_0045.02_post_itsc_12turn.csv</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>itsc_4turn_halfload</t>
+          <t>itsc_12turn</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>0.059549</v>
+        <v>0.222124</v>
       </c>
       <c r="E128" t="n">
-        <v>0.05955</v>
+        <v>0.22212</v>
       </c>
       <c r="F128">
         <f>(D128/E128-1)*100</f>
@@ -8552,6 +8558,1463 @@
       </c>
       <c r="G128">
         <f>IF(ABS(F128)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>waveform_0045.02_pre_itsc_4turn.csv</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>itsc_4turn</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>0.031298</v>
+      </c>
+      <c r="E129" t="n">
+        <v>0.0313</v>
+      </c>
+      <c r="F129">
+        <f>(D129/E129-1)*100</f>
+        <v/>
+      </c>
+      <c r="G129">
+        <f>IF(ABS(F129)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>waveform_0045.05_post_itsc_12turn.csv</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>itsc_12turn</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>0.222124</v>
+      </c>
+      <c r="E130" t="n">
+        <v>0.22212</v>
+      </c>
+      <c r="F130">
+        <f>(D130/E130-1)*100</f>
+        <v/>
+      </c>
+      <c r="G130">
+        <f>IF(ABS(F130)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>waveform_0045.05_pre_itsc_4turn.csv</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>itsc_4turn</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>0.031298</v>
+      </c>
+      <c r="E131" t="n">
+        <v>0.0313</v>
+      </c>
+      <c r="F131">
+        <f>(D131/E131-1)*100</f>
+        <v/>
+      </c>
+      <c r="G131">
+        <f>IF(ABS(F131)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>waveform_0075.02_post_overload.csv</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>overload</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="E132" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F132">
+        <f>(D132/E132-1)*100</f>
+        <v/>
+      </c>
+      <c r="G132">
+        <f>IF(ABS(F132)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>waveform_0075.02_pre_itsc_12turn.csv</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>itsc_12turn</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>0.222124</v>
+      </c>
+      <c r="E133" t="n">
+        <v>0.22212</v>
+      </c>
+      <c r="F133">
+        <f>(D133/E133-1)*100</f>
+        <v/>
+      </c>
+      <c r="G133">
+        <f>IF(ABS(F133)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>waveform_0075.05_post_overload.csv</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>overload</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="E134" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F134">
+        <f>(D134/E134-1)*100</f>
+        <v/>
+      </c>
+      <c r="G134">
+        <f>IF(ABS(F134)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>waveform_0075.05_pre_itsc_12turn.csv</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>itsc_12turn</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>0.222124</v>
+      </c>
+      <c r="E135" t="n">
+        <v>0.22212</v>
+      </c>
+      <c r="F135">
+        <f>(D135/E135-1)*100</f>
+        <v/>
+      </c>
+      <c r="G135">
+        <f>IF(ABS(F135)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>waveform_0095.02_post_voltage_unbalance.csv</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>voltage_unbalance</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>0.059508</v>
+      </c>
+      <c r="E136" t="n">
+        <v>0.05951</v>
+      </c>
+      <c r="F136">
+        <f>(D136/E136-1)*100</f>
+        <v/>
+      </c>
+      <c r="G136">
+        <f>IF(ABS(F136)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>waveform_0095.02_pre_overload.csv</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>overload</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F137">
+        <f>(D137/E137-1)*100</f>
+        <v/>
+      </c>
+      <c r="G137">
+        <f>IF(ABS(F137)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>waveform_0120.03_post_single_phasing.csv</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>single_phasing</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>0.479167</v>
+      </c>
+      <c r="E138" t="n">
+        <v>0.47917</v>
+      </c>
+      <c r="F138">
+        <f>(D138/E138-1)*100</f>
+        <v/>
+      </c>
+      <c r="G138">
+        <f>IF(ABS(F138)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>waveform_0120.03_pre_voltage_unbalance.csv</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>voltage_unbalance</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>0.059508</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0.05951</v>
+      </c>
+      <c r="F139">
+        <f>(D139/E139-1)*100</f>
+        <v/>
+      </c>
+      <c r="G139">
+        <f>IF(ABS(F139)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>waveform_0120.04_post_single_phasing.csv</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>single_phasing</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>0.479167</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0.47917</v>
+      </c>
+      <c r="F140">
+        <f>(D140/E140-1)*100</f>
+        <v/>
+      </c>
+      <c r="G140">
+        <f>IF(ABS(F140)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>waveform_0120.04_pre_voltage_unbalance.csv</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>voltage_unbalance</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>0.059508</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0.05951</v>
+      </c>
+      <c r="F141">
+        <f>(D141/E141-1)*100</f>
+        <v/>
+      </c>
+      <c r="G141">
+        <f>IF(ABS(F141)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>waveform_0120.05_post_single_phasing.csv</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>single_phasing</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>0.479167</v>
+      </c>
+      <c r="E142" t="n">
+        <v>0.47917</v>
+      </c>
+      <c r="F142">
+        <f>(D142/E142-1)*100</f>
+        <v/>
+      </c>
+      <c r="G142">
+        <f>IF(ABS(F142)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>waveform_0120.05_pre_voltage_unbalance.csv</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>voltage_unbalance</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>0.059508</v>
+      </c>
+      <c r="E143" t="n">
+        <v>0.05951</v>
+      </c>
+      <c r="F143">
+        <f>(D143/E143-1)*100</f>
+        <v/>
+      </c>
+      <c r="G143">
+        <f>IF(ABS(F143)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>waveform_0145.02_post_no_load.csv</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>no_load</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="E144" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F144">
+        <f>(D144/E144-1)*100</f>
+        <v/>
+      </c>
+      <c r="G144">
+        <f>IF(ABS(F144)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>waveform_0145.02_pre_single_phasing.csv</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>single_phasing</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>0.479167</v>
+      </c>
+      <c r="E145" t="n">
+        <v>0.47917</v>
+      </c>
+      <c r="F145">
+        <f>(D145/E145-1)*100</f>
+        <v/>
+      </c>
+      <c r="G145">
+        <f>IF(ABS(F145)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>waveform_0145.05_post_no_load.csv</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>no_load</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="E146" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F146">
+        <f>(D146/E146-1)*100</f>
+        <v/>
+      </c>
+      <c r="G146">
+        <f>IF(ABS(F146)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>waveform_0145.05_pre_single_phasing.csv</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>single_phasing</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>0.479167</v>
+      </c>
+      <c r="E147" t="n">
+        <v>0.47917</v>
+      </c>
+      <c r="F147">
+        <f>(D147/E147-1)*100</f>
+        <v/>
+      </c>
+      <c r="G147">
+        <f>IF(ABS(F147)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>waveform_0145.06_post_no_load.csv</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>no_load</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="E148" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F148">
+        <f>(D148/E148-1)*100</f>
+        <v/>
+      </c>
+      <c r="G148">
+        <f>IF(ABS(F148)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>waveform_0145.06_pre_single_phasing.csv</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>single_phasing</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>0.479167</v>
+      </c>
+      <c r="E149" t="n">
+        <v>0.47917</v>
+      </c>
+      <c r="F149">
+        <f>(D149/E149-1)*100</f>
+        <v/>
+      </c>
+      <c r="G149">
+        <f>IF(ABS(F149)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>waveform_0165.03_post_itsc_8turn.csv</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>itsc_8turn</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>0.122089</v>
+      </c>
+      <c r="E150" t="n">
+        <v>0.12209</v>
+      </c>
+      <c r="F150">
+        <f>(D150/E150-1)*100</f>
+        <v/>
+      </c>
+      <c r="G150">
+        <f>IF(ABS(F150)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>waveform_0165.03_pre_no_load.csv</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>no_load</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="E151" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F151">
+        <f>(D151/E151-1)*100</f>
+        <v/>
+      </c>
+      <c r="G151">
+        <f>IF(ABS(F151)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>waveform_0165.04_post_itsc_8turn.csv</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>itsc_8turn</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>0.122089</v>
+      </c>
+      <c r="E152" t="n">
+        <v>0.12209</v>
+      </c>
+      <c r="F152">
+        <f>(D152/E152-1)*100</f>
+        <v/>
+      </c>
+      <c r="G152">
+        <f>IF(ABS(F152)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>waveform_0165.04_pre_no_load.csv</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>no_load</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="E153" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F153">
+        <f>(D153/E153-1)*100</f>
+        <v/>
+      </c>
+      <c r="G153">
+        <f>IF(ABS(F153)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>waveform_0165.06_post_itsc_8turn.csv</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>itsc_8turn</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>0.122089</v>
+      </c>
+      <c r="E154" t="n">
+        <v>0.12209</v>
+      </c>
+      <c r="F154">
+        <f>(D154/E154-1)*100</f>
+        <v/>
+      </c>
+      <c r="G154">
+        <f>IF(ABS(F154)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>waveform_0165.06_pre_no_load.csv</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>no_load</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="E155" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F155">
+        <f>(D155/E155-1)*100</f>
+        <v/>
+      </c>
+      <c r="G155">
+        <f>IF(ABS(F155)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>waveform_0185.03_post_itsc_16turn.csv</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>itsc_16turn</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>0.313563</v>
+      </c>
+      <c r="E156" t="n">
+        <v>0.31356</v>
+      </c>
+      <c r="F156">
+        <f>(D156/E156-1)*100</f>
+        <v/>
+      </c>
+      <c r="G156">
+        <f>IF(ABS(F156)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>waveform_0185.03_pre_itsc_8turn.csv</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>itsc_8turn</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>0.122089</v>
+      </c>
+      <c r="E157" t="n">
+        <v>0.12209</v>
+      </c>
+      <c r="F157">
+        <f>(D157/E157-1)*100</f>
+        <v/>
+      </c>
+      <c r="G157">
+        <f>IF(ABS(F157)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>waveform_0185.05_post_itsc_16turn.csv</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>itsc_16turn</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>0.313563</v>
+      </c>
+      <c r="E158" t="n">
+        <v>0.31356</v>
+      </c>
+      <c r="F158">
+        <f>(D158/E158-1)*100</f>
+        <v/>
+      </c>
+      <c r="G158">
+        <f>IF(ABS(F158)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>waveform_0185.05_pre_itsc_8turn.csv</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>itsc_8turn</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>0.122089</v>
+      </c>
+      <c r="E159" t="n">
+        <v>0.12209</v>
+      </c>
+      <c r="F159">
+        <f>(D159/E159-1)*100</f>
+        <v/>
+      </c>
+      <c r="G159">
+        <f>IF(ABS(F159)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>waveform_0205.00_post_itsc_4turn_resistive.csv</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>itsc_4turn_resistive</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>0.022165</v>
+      </c>
+      <c r="E160" t="n">
+        <v>0.02217</v>
+      </c>
+      <c r="F160">
+        <f>(D160/E160-1)*100</f>
+        <v/>
+      </c>
+      <c r="G160">
+        <f>IF(ABS(F160)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>waveform_0205.00_pre_itsc_16turn.csv</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>itsc_16turn</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>0.313563</v>
+      </c>
+      <c r="E161" t="n">
+        <v>0.31356</v>
+      </c>
+      <c r="F161">
+        <f>(D161/E161-1)*100</f>
+        <v/>
+      </c>
+      <c r="G161">
+        <f>IF(ABS(F161)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>waveform_0205.04_post_itsc_4turn_resistive.csv</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>itsc_4turn_resistive</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>0.022165</v>
+      </c>
+      <c r="E162" t="n">
+        <v>0.02217</v>
+      </c>
+      <c r="F162">
+        <f>(D162/E162-1)*100</f>
+        <v/>
+      </c>
+      <c r="G162">
+        <f>IF(ABS(F162)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>waveform_0205.04_pre_itsc_16turn.csv</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>itsc_16turn</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>0.313563</v>
+      </c>
+      <c r="E163" t="n">
+        <v>0.31356</v>
+      </c>
+      <c r="F163">
+        <f>(D163/E163-1)*100</f>
+        <v/>
+      </c>
+      <c r="G163">
+        <f>IF(ABS(F163)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>waveform_0225.00_post_itsc_4turn_halfload.csv</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>itsc_4turn_halfload</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="E164" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="F164">
+        <f>(D164/E164-1)*100</f>
+        <v/>
+      </c>
+      <c r="G164">
+        <f>IF(ABS(F164)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>waveform_0225.00_pre_itsc_4turn_resistive.csv</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>itsc_4turn_resistive</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>0.022165</v>
+      </c>
+      <c r="E165" t="n">
+        <v>0.02217</v>
+      </c>
+      <c r="F165">
+        <f>(D165/E165-1)*100</f>
+        <v/>
+      </c>
+      <c r="G165">
+        <f>IF(ABS(F165)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>waveform_0225.02_post_itsc_4turn_halfload.csv</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>itsc_4turn_halfload</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="E166" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="F166">
+        <f>(D166/E166-1)*100</f>
+        <v/>
+      </c>
+      <c r="G166">
+        <f>IF(ABS(F166)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>waveform_0225.02_pre_itsc_4turn_resistive.csv</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>itsc_4turn_resistive</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>0.022165</v>
+      </c>
+      <c r="E167" t="n">
+        <v>0.02217</v>
+      </c>
+      <c r="F167">
+        <f>(D167/E167-1)*100</f>
+        <v/>
+      </c>
+      <c r="G167">
+        <f>IF(ABS(F167)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>waveform_0225.03_post_itsc_4turn_halfload.csv</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>itsc_4turn_halfload</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>0.059549</v>
+      </c>
+      <c r="E168" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="F168">
+        <f>(D168/E168-1)*100</f>
+        <v/>
+      </c>
+      <c r="G168">
+        <f>IF(ABS(F168)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>waveform_0225.03_pre_itsc_4turn_resistive.csv</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>itsc_4turn_resistive</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>0.022165</v>
+      </c>
+      <c r="E169" t="n">
+        <v>0.02217</v>
+      </c>
+      <c r="F169">
+        <f>(D169/E169-1)*100</f>
+        <v/>
+      </c>
+      <c r="G169">
+        <f>IF(ABS(F169)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>waveform_0245.02_post_itsc_4turn_halfload.csv</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>itsc_4turn_halfload</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="E170" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="F170">
+        <f>(D170/E170-1)*100</f>
+        <v/>
+      </c>
+      <c r="G170">
+        <f>IF(ABS(F170)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>waveform_0245.02_pre_itsc_4turn_halfload.csv</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>itsc_4turn_halfload</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="E171" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="F171">
+        <f>(D171/E171-1)*100</f>
+        <v/>
+      </c>
+      <c r="G171">
+        <f>IF(ABS(F171)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>waveform_0245.04_post_itsc_4turn_halfload.csv</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>itsc_4turn_halfload</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>0.059549</v>
+      </c>
+      <c r="E172" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="F172">
+        <f>(D172/E172-1)*100</f>
+        <v/>
+      </c>
+      <c r="G172">
+        <f>IF(ABS(F172)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>waveform_0245.04_pre_itsc_4turn_halfload.csv</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>itsc_4turn_halfload</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>0.059549</v>
+      </c>
+      <c r="E173" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="F173">
+        <f>(D173/E173-1)*100</f>
+        <v/>
+      </c>
+      <c r="G173">
+        <f>IF(ABS(F173)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>waveform_0245.05_post_itsc_4turn_halfload.csv</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>itsc_4turn_halfload</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="E174" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="F174">
+        <f>(D174/E174-1)*100</f>
+        <v/>
+      </c>
+      <c r="G174">
+        <f>IF(ABS(F174)&lt;=0.5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>a180</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>waveform_0245.05_pre_itsc_4turn_halfload.csv</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>itsc_4turn_halfload</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="E175" t="n">
+        <v>0.05955</v>
+      </c>
+      <c r="F175">
+        <f>(D175/E175-1)*100</f>
+        <v/>
+      </c>
+      <c r="G175">
+        <f>IF(ABS(F175)&lt;=0.5,"PASS","FAIL")</f>
         <v/>
       </c>
     </row>

</xml_diff>